<commit_message>
Cap nhat chuan hoa so lieu 03-3-2026
</commit_message>
<xml_diff>
--- a/Chuẩn hóa giao thong.xlsx
+++ b/Chuẩn hóa giao thong.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\@Giaothong2\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\@Giaothong2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85F461E6-524C-40FE-B601-AE25A497307E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{491C02DA-631E-4526-9E55-0AB35EF134D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30612" yWindow="-6000" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Phụ Lục 1" sheetId="1" r:id="rId1"/>
@@ -5890,36 +5890,6 @@
     <xf numFmtId="2" fontId="35" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5991,6 +5961,36 @@
     </xf>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="14">
@@ -6384,7 +6384,7 @@
     <col min="11" max="11" width="19.3984375" style="5" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="32.59765625" style="5" customWidth="1"/>
     <col min="13" max="13" width="20.59765625" style="5" customWidth="1"/>
-    <col min="14" max="14" width="94.59765625" style="199" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="94.59765625" style="189" bestFit="1" customWidth="1"/>
     <col min="15" max="16384" width="9" style="5"/>
   </cols>
   <sheetData>
@@ -6428,7 +6428,7 @@
       <c r="M1" s="150" t="s">
         <v>1594</v>
       </c>
-      <c r="N1" s="187" t="s">
+      <c r="N1" s="177" t="s">
         <v>1579</v>
       </c>
     </row>
@@ -6450,7 +6450,7 @@
       <c r="K2" s="150"/>
       <c r="L2" s="150"/>
       <c r="M2" s="150"/>
-      <c r="N2" s="187"/>
+      <c r="N2" s="177"/>
     </row>
     <row r="3" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="131" t="s">
@@ -6474,7 +6474,7 @@
       <c r="K3" s="149"/>
       <c r="L3" s="149"/>
       <c r="M3" s="149"/>
-      <c r="N3" s="188"/>
+      <c r="N3" s="178"/>
     </row>
     <row r="4" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9">
@@ -6510,7 +6510,7 @@
       <c r="M4" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N4" s="189" t="s">
+      <c r="N4" s="179" t="s">
         <v>973</v>
       </c>
     </row>
@@ -6546,7 +6546,7 @@
       <c r="M5" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N5" s="189" t="s">
+      <c r="N5" s="179" t="s">
         <v>974</v>
       </c>
     </row>
@@ -6582,7 +6582,7 @@
       <c r="M6" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N6" s="189" t="s">
+      <c r="N6" s="179" t="s">
         <v>976</v>
       </c>
     </row>
@@ -6618,7 +6618,7 @@
       <c r="M7" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N7" s="189" t="s">
+      <c r="N7" s="179" t="s">
         <v>974</v>
       </c>
     </row>
@@ -6656,7 +6656,7 @@
       <c r="M8" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N8" s="189" t="s">
+      <c r="N8" s="179" t="s">
         <v>978</v>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
       <c r="K9" s="6"/>
       <c r="L9" s="6"/>
       <c r="M9" s="6"/>
-      <c r="N9" s="190"/>
+      <c r="N9" s="180"/>
     </row>
     <row r="10" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="26">
@@ -6718,7 +6718,7 @@
       <c r="M10" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N10" s="189" t="s">
+      <c r="N10" s="179" t="s">
         <v>1021</v>
       </c>
     </row>
@@ -6754,7 +6754,7 @@
       <c r="M11" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N11" s="189" t="s">
+      <c r="N11" s="179" t="s">
         <v>1023</v>
       </c>
     </row>
@@ -6790,7 +6790,7 @@
       <c r="M12" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N12" s="189" t="s">
+      <c r="N12" s="179" t="s">
         <v>1021</v>
       </c>
     </row>
@@ -6826,7 +6826,7 @@
       <c r="M13" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N13" s="189" t="s">
+      <c r="N13" s="179" t="s">
         <v>1023</v>
       </c>
     </row>
@@ -6850,14 +6850,14 @@
       <c r="I14" s="165"/>
       <c r="J14" s="166"/>
       <c r="K14" s="163"/>
-      <c r="L14" s="191" t="str">
+      <c r="L14" s="181" t="str">
         <f>N14</f>
         <v>Đi chung Quốc lộ 70</v>
       </c>
       <c r="M14" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N14" s="188" t="s">
+      <c r="N14" s="178" t="s">
         <v>1583</v>
       </c>
     </row>
@@ -6891,11 +6891,11 @@
       <c r="K15" s="6">
         <v>5.5</v>
       </c>
-      <c r="L15" s="191"/>
+      <c r="L15" s="181"/>
       <c r="M15" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N15" s="189" t="s">
+      <c r="N15" s="179" t="s">
         <v>1027</v>
       </c>
     </row>
@@ -6919,9 +6919,9 @@
       </c>
       <c r="J16" s="77"/>
       <c r="K16" s="6"/>
-      <c r="L16" s="191"/>
-      <c r="M16" s="191"/>
-      <c r="N16" s="188"/>
+      <c r="L16" s="181"/>
+      <c r="M16" s="181"/>
+      <c r="N16" s="178"/>
     </row>
     <row r="17" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
@@ -6949,11 +6949,11 @@
       </c>
       <c r="J17" s="77"/>
       <c r="K17" s="6"/>
-      <c r="L17" s="191"/>
-      <c r="M17" s="191" t="s">
+      <c r="L17" s="181"/>
+      <c r="M17" s="181" t="s">
         <v>1596</v>
       </c>
-      <c r="N17" s="192" t="s">
+      <c r="N17" s="182" t="s">
         <v>283</v>
       </c>
     </row>
@@ -6985,11 +6985,11 @@
       <c r="K18" s="6">
         <v>6.5</v>
       </c>
-      <c r="L18" s="192"/>
-      <c r="M18" s="192" t="s">
+      <c r="L18" s="182"/>
+      <c r="M18" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N18" s="189" t="s">
+      <c r="N18" s="179" t="s">
         <v>1079</v>
       </c>
     </row>
@@ -7017,11 +7017,11 @@
       </c>
       <c r="J19" s="77"/>
       <c r="K19" s="6"/>
-      <c r="L19" s="191"/>
-      <c r="M19" s="191" t="s">
+      <c r="L19" s="181"/>
+      <c r="M19" s="181" t="s">
         <v>1596</v>
       </c>
-      <c r="N19" s="192" t="s">
+      <c r="N19" s="182" t="s">
         <v>283</v>
       </c>
     </row>
@@ -7053,11 +7053,11 @@
       <c r="K20" s="6">
         <v>6.5</v>
       </c>
-      <c r="L20" s="192"/>
-      <c r="M20" s="192" t="s">
+      <c r="L20" s="182"/>
+      <c r="M20" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N20" s="189" t="s">
+      <c r="N20" s="179" t="s">
         <v>1080</v>
       </c>
     </row>
@@ -7081,12 +7081,12 @@
       <c r="I21" s="172"/>
       <c r="J21" s="166"/>
       <c r="K21" s="163"/>
-      <c r="L21" s="192" t="str">
+      <c r="L21" s="182" t="str">
         <f>N21</f>
         <v>Đi chung với QL.70</v>
       </c>
-      <c r="M21" s="192"/>
-      <c r="N21" s="188" t="s">
+      <c r="M21" s="182"/>
+      <c r="N21" s="178" t="s">
         <v>1584</v>
       </c>
     </row>
@@ -7118,11 +7118,11 @@
       <c r="K22" s="6">
         <v>11</v>
       </c>
-      <c r="L22" s="192"/>
-      <c r="M22" s="192" t="s">
+      <c r="L22" s="182"/>
+      <c r="M22" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N22" s="193" t="s">
+      <c r="N22" s="183" t="s">
         <v>882</v>
       </c>
     </row>
@@ -7154,11 +7154,11 @@
       <c r="K23" s="6">
         <v>6.5</v>
       </c>
-      <c r="L23" s="196"/>
-      <c r="M23" s="192" t="s">
+      <c r="L23" s="186"/>
+      <c r="M23" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N23" s="193" t="s">
+      <c r="N23" s="183" t="s">
         <v>880</v>
       </c>
     </row>
@@ -7190,11 +7190,11 @@
       <c r="K24" s="6" t="s">
         <v>1265</v>
       </c>
-      <c r="L24" s="191"/>
-      <c r="M24" s="192" t="s">
+      <c r="L24" s="181"/>
+      <c r="M24" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N24" s="193" t="s">
+      <c r="N24" s="183" t="s">
         <v>854</v>
       </c>
     </row>
@@ -7226,11 +7226,11 @@
       <c r="K25" s="6">
         <v>6.5</v>
       </c>
-      <c r="L25" s="191"/>
-      <c r="M25" s="192" t="s">
+      <c r="L25" s="181"/>
+      <c r="M25" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N25" s="193" t="s">
+      <c r="N25" s="183" t="s">
         <v>880</v>
       </c>
     </row>
@@ -7263,10 +7263,10 @@
         <v>11</v>
       </c>
       <c r="L26" s="6"/>
-      <c r="M26" s="192" t="s">
+      <c r="M26" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N26" s="193" t="s">
+      <c r="N26" s="183" t="s">
         <v>882</v>
       </c>
     </row>
@@ -7299,10 +7299,10 @@
         <v>6.5</v>
       </c>
       <c r="L27" s="6"/>
-      <c r="M27" s="192" t="s">
+      <c r="M27" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N27" s="193" t="s">
+      <c r="N27" s="183" t="s">
         <v>880</v>
       </c>
     </row>
@@ -7335,10 +7335,10 @@
         <v>6.5</v>
       </c>
       <c r="L28" s="6"/>
-      <c r="M28" s="192" t="s">
+      <c r="M28" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N28" s="193" t="s">
+      <c r="N28" s="183" t="s">
         <v>1138</v>
       </c>
     </row>
@@ -7371,10 +7371,10 @@
         <v>1263</v>
       </c>
       <c r="L29" s="6"/>
-      <c r="M29" s="192" t="s">
+      <c r="M29" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N29" s="193" t="s">
+      <c r="N29" s="183" t="s">
         <v>852</v>
       </c>
     </row>
@@ -7407,10 +7407,10 @@
         <v>30</v>
       </c>
       <c r="L30" s="6"/>
-      <c r="M30" s="192" t="s">
+      <c r="M30" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N30" s="193" t="s">
+      <c r="N30" s="183" t="s">
         <v>881</v>
       </c>
     </row>
@@ -7443,10 +7443,10 @@
         <v>30</v>
       </c>
       <c r="L31" s="6"/>
-      <c r="M31" s="192" t="s">
+      <c r="M31" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N31" s="193" t="s">
+      <c r="N31" s="183" t="s">
         <v>1170</v>
       </c>
     </row>
@@ -7479,10 +7479,10 @@
         <v>30</v>
       </c>
       <c r="L32" s="6"/>
-      <c r="M32" s="192" t="s">
+      <c r="M32" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N32" s="193" t="s">
+      <c r="N32" s="183" t="s">
         <v>881</v>
       </c>
     </row>
@@ -7510,10 +7510,10 @@
         <f>N33</f>
         <v>Đi chung với QL.4D</v>
       </c>
-      <c r="M33" s="192" t="s">
+      <c r="M33" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N33" s="188" t="s">
+      <c r="N33" s="178" t="s">
         <v>1585</v>
       </c>
     </row>
@@ -7546,10 +7546,10 @@
         <v>11</v>
       </c>
       <c r="L34" s="6"/>
-      <c r="M34" s="192" t="s">
+      <c r="M34" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N34" s="193" t="s">
+      <c r="N34" s="183" t="s">
         <v>882</v>
       </c>
     </row>
@@ -7582,10 +7582,10 @@
         <v>9.5</v>
       </c>
       <c r="L35" s="6"/>
-      <c r="M35" s="192" t="s">
+      <c r="M35" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N35" s="193" t="s">
+      <c r="N35" s="183" t="s">
         <v>1146</v>
       </c>
     </row>
@@ -7615,10 +7615,10 @@
         <v>14</v>
       </c>
       <c r="L36" s="6"/>
-      <c r="M36" s="192" t="s">
+      <c r="M36" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N36" s="193" t="s">
+      <c r="N36" s="183" t="s">
         <v>1148</v>
       </c>
     </row>
@@ -7653,10 +7653,10 @@
         <v>5.5</v>
       </c>
       <c r="L37" s="6"/>
-      <c r="M37" s="192" t="s">
+      <c r="M37" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N37" s="189" t="s">
+      <c r="N37" s="179" t="s">
         <v>1150</v>
       </c>
     </row>
@@ -7681,8 +7681,8 @@
       <c r="J38" s="77"/>
       <c r="K38" s="6"/>
       <c r="L38" s="6"/>
-      <c r="M38" s="192"/>
-      <c r="N38" s="188"/>
+      <c r="M38" s="182"/>
+      <c r="N38" s="178"/>
     </row>
     <row r="39" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
@@ -7715,10 +7715,10 @@
         <v>1263</v>
       </c>
       <c r="L39" s="6"/>
-      <c r="M39" s="192" t="s">
+      <c r="M39" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N39" s="193" t="s">
+      <c r="N39" s="183" t="s">
         <v>852</v>
       </c>
     </row>
@@ -7751,10 +7751,10 @@
         <v>1265</v>
       </c>
       <c r="L40" s="6"/>
-      <c r="M40" s="192" t="s">
+      <c r="M40" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N40" s="193" t="s">
+      <c r="N40" s="183" t="s">
         <v>854</v>
       </c>
     </row>
@@ -7787,10 +7787,10 @@
         <v>1264</v>
       </c>
       <c r="L41" s="6"/>
-      <c r="M41" s="192" t="s">
+      <c r="M41" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N41" s="193" t="s">
+      <c r="N41" s="183" t="s">
         <v>856</v>
       </c>
     </row>
@@ -7823,10 +7823,10 @@
         <v>1263</v>
       </c>
       <c r="L42" s="6"/>
-      <c r="M42" s="192" t="s">
+      <c r="M42" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N42" s="193" t="s">
+      <c r="N42" s="183" t="s">
         <v>852</v>
       </c>
     </row>
@@ -7859,10 +7859,10 @@
         <v>1263</v>
       </c>
       <c r="L43" s="6"/>
-      <c r="M43" s="192" t="s">
+      <c r="M43" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N43" s="193" t="s">
+      <c r="N43" s="183" t="s">
         <v>859</v>
       </c>
     </row>
@@ -7895,10 +7895,10 @@
         <v>1263</v>
       </c>
       <c r="L44" s="6"/>
-      <c r="M44" s="192" t="s">
+      <c r="M44" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N44" s="193" t="s">
+      <c r="N44" s="183" t="s">
         <v>852</v>
       </c>
     </row>
@@ -7931,10 +7931,10 @@
         <v>1263</v>
       </c>
       <c r="L45" s="6"/>
-      <c r="M45" s="192" t="s">
+      <c r="M45" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N45" s="193" t="s">
+      <c r="N45" s="183" t="s">
         <v>859</v>
       </c>
     </row>
@@ -7967,10 +7967,10 @@
         <v>1263</v>
       </c>
       <c r="L46" s="6"/>
-      <c r="M46" s="192" t="s">
+      <c r="M46" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N46" s="193" t="s">
+      <c r="N46" s="183" t="s">
         <v>852</v>
       </c>
     </row>
@@ -8003,10 +8003,10 @@
         <v>1263</v>
       </c>
       <c r="L47" s="6"/>
-      <c r="M47" s="192" t="s">
+      <c r="M47" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N47" s="193" t="s">
+      <c r="N47" s="183" t="s">
         <v>859</v>
       </c>
     </row>
@@ -8039,10 +8039,10 @@
         <v>1263</v>
       </c>
       <c r="L48" s="6"/>
-      <c r="M48" s="192" t="s">
+      <c r="M48" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N48" s="193" t="s">
+      <c r="N48" s="183" t="s">
         <v>852</v>
       </c>
     </row>
@@ -8075,10 +8075,10 @@
         <v>1263</v>
       </c>
       <c r="L49" s="6"/>
-      <c r="M49" s="192" t="s">
+      <c r="M49" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N49" s="193" t="s">
+      <c r="N49" s="183" t="s">
         <v>852</v>
       </c>
     </row>
@@ -8111,10 +8111,10 @@
         <v>1263</v>
       </c>
       <c r="L50" s="6"/>
-      <c r="M50" s="192" t="s">
+      <c r="M50" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N50" s="193" t="s">
+      <c r="N50" s="183" t="s">
         <v>859</v>
       </c>
     </row>
@@ -8147,10 +8147,10 @@
         <v>1263</v>
       </c>
       <c r="L51" s="6"/>
-      <c r="M51" s="192" t="s">
+      <c r="M51" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N51" s="193" t="s">
+      <c r="N51" s="183" t="s">
         <v>852</v>
       </c>
     </row>
@@ -8183,10 +8183,10 @@
         <v>1263</v>
       </c>
       <c r="L52" s="6"/>
-      <c r="M52" s="192" t="s">
+      <c r="M52" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N52" s="193" t="s">
+      <c r="N52" s="183" t="s">
         <v>852</v>
       </c>
     </row>
@@ -8221,10 +8221,10 @@
         <v>1263</v>
       </c>
       <c r="L53" s="6"/>
-      <c r="M53" s="192" t="s">
+      <c r="M53" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N53" s="193" t="s">
+      <c r="N53" s="183" t="s">
         <v>852</v>
       </c>
     </row>
@@ -8250,7 +8250,7 @@
       <c r="K54" s="6"/>
       <c r="L54" s="6"/>
       <c r="M54" s="6"/>
-      <c r="N54" s="188"/>
+      <c r="N54" s="178"/>
     </row>
     <row r="55" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="24">
@@ -8283,10 +8283,10 @@
         <v>5.5</v>
       </c>
       <c r="L55" s="6"/>
-      <c r="M55" s="192" t="s">
+      <c r="M55" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N55" s="193" t="s">
+      <c r="N55" s="183" t="s">
         <v>786</v>
       </c>
     </row>
@@ -8318,10 +8318,10 @@
         <v>9</v>
       </c>
       <c r="L56" s="6"/>
-      <c r="M56" s="192" t="s">
+      <c r="M56" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N56" s="193" t="s">
+      <c r="N56" s="183" t="s">
         <v>810</v>
       </c>
     </row>
@@ -8354,10 +8354,10 @@
         <v>5.5</v>
       </c>
       <c r="L57" s="6"/>
-      <c r="M57" s="192" t="s">
+      <c r="M57" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N57" s="193" t="s">
+      <c r="N57" s="183" t="s">
         <v>786</v>
       </c>
     </row>
@@ -8390,10 +8390,10 @@
         <v>9</v>
       </c>
       <c r="L58" s="6"/>
-      <c r="M58" s="192" t="s">
+      <c r="M58" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N58" s="193" t="s">
+      <c r="N58" s="183" t="s">
         <v>810</v>
       </c>
     </row>
@@ -8426,10 +8426,10 @@
         <v>10.5</v>
       </c>
       <c r="L59" s="6"/>
-      <c r="M59" s="192" t="s">
+      <c r="M59" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N59" s="193" t="s">
+      <c r="N59" s="183" t="s">
         <v>1157</v>
       </c>
     </row>
@@ -8462,10 +8462,10 @@
         <v>10.5</v>
       </c>
       <c r="L60" s="6"/>
-      <c r="M60" s="192" t="s">
+      <c r="M60" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N60" s="193" t="s">
+      <c r="N60" s="183" t="s">
         <v>1159</v>
       </c>
     </row>
@@ -8498,10 +8498,10 @@
         <v>5.5</v>
       </c>
       <c r="L61" s="6"/>
-      <c r="M61" s="192" t="s">
+      <c r="M61" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N61" s="193" t="s">
+      <c r="N61" s="183" t="s">
         <v>786</v>
       </c>
     </row>
@@ -8534,10 +8534,10 @@
         <v>5.5</v>
       </c>
       <c r="L62" s="6"/>
-      <c r="M62" s="192" t="s">
+      <c r="M62" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N62" s="193" t="s">
+      <c r="N62" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -8570,10 +8570,10 @@
         <v>9</v>
       </c>
       <c r="L63" s="6"/>
-      <c r="M63" s="192" t="s">
+      <c r="M63" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N63" s="193" t="s">
+      <c r="N63" s="183" t="s">
         <v>810</v>
       </c>
     </row>
@@ -8606,10 +8606,10 @@
         <v>5.5</v>
       </c>
       <c r="L64" s="6"/>
-      <c r="M64" s="192" t="s">
+      <c r="M64" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N64" s="193" t="s">
+      <c r="N64" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -8642,10 +8642,10 @@
         <v>9</v>
       </c>
       <c r="L65" s="6"/>
-      <c r="M65" s="192" t="s">
+      <c r="M65" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N65" s="193" t="s">
+      <c r="N65" s="183" t="s">
         <v>810</v>
       </c>
     </row>
@@ -8680,10 +8680,10 @@
         <v>5.5</v>
       </c>
       <c r="L66" s="6"/>
-      <c r="M66" s="192" t="s">
+      <c r="M66" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N66" s="193" t="s">
+      <c r="N66" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -8709,7 +8709,7 @@
       <c r="K67" s="6"/>
       <c r="L67" s="6"/>
       <c r="M67" s="6"/>
-      <c r="N67" s="188"/>
+      <c r="N67" s="178"/>
     </row>
     <row r="68" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="20">
@@ -8742,10 +8742,10 @@
         <v>5.5</v>
       </c>
       <c r="L68" s="6"/>
-      <c r="M68" s="192" t="s">
+      <c r="M68" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N68" s="193" t="s">
+      <c r="N68" s="183" t="s">
         <v>285</v>
       </c>
     </row>
@@ -8778,10 +8778,10 @@
         <v>5.5</v>
       </c>
       <c r="L69" s="6"/>
-      <c r="M69" s="192" t="s">
+      <c r="M69" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N69" s="193" t="s">
+      <c r="N69" s="183" t="s">
         <v>870</v>
       </c>
     </row>
@@ -8814,10 +8814,10 @@
         <v>1267</v>
       </c>
       <c r="L70" s="6"/>
-      <c r="M70" s="192" t="s">
+      <c r="M70" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N70" s="193" t="s">
+      <c r="N70" s="183" t="s">
         <v>872</v>
       </c>
     </row>
@@ -8850,10 +8850,10 @@
         <v>11</v>
       </c>
       <c r="L71" s="6"/>
-      <c r="M71" s="192" t="s">
+      <c r="M71" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N71" s="193" t="s">
+      <c r="N71" s="183" t="s">
         <v>874</v>
       </c>
     </row>
@@ -8886,10 +8886,10 @@
         <v>1169</v>
       </c>
       <c r="L72" s="6"/>
-      <c r="M72" s="192" t="s">
+      <c r="M72" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N72" s="193" t="s">
+      <c r="N72" s="183" t="s">
         <v>876</v>
       </c>
     </row>
@@ -8924,10 +8924,10 @@
         <v>12</v>
       </c>
       <c r="L73" s="6"/>
-      <c r="M73" s="192" t="s">
+      <c r="M73" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N73" s="193" t="s">
+      <c r="N73" s="183" t="s">
         <v>878</v>
       </c>
     </row>
@@ -8953,7 +8953,7 @@
       <c r="K74" s="6"/>
       <c r="L74" s="6"/>
       <c r="M74" s="6"/>
-      <c r="N74" s="188"/>
+      <c r="N74" s="178"/>
     </row>
     <row r="75" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="24">
@@ -8986,10 +8986,10 @@
         <v>7.5</v>
       </c>
       <c r="L75" s="6"/>
-      <c r="M75" s="192" t="s">
+      <c r="M75" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N75" s="193" t="s">
+      <c r="N75" s="183" t="s">
         <v>784</v>
       </c>
     </row>
@@ -9023,10 +9023,10 @@
         <v>5.5</v>
       </c>
       <c r="L76" s="6"/>
-      <c r="M76" s="192" t="s">
+      <c r="M76" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N76" s="193" t="s">
+      <c r="N76" s="183" t="s">
         <v>786</v>
       </c>
     </row>
@@ -9052,7 +9052,7 @@
       <c r="K77" s="6"/>
       <c r="L77" s="6"/>
       <c r="M77" s="6"/>
-      <c r="N77" s="188"/>
+      <c r="N77" s="178"/>
     </row>
     <row r="78" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="24">
@@ -9085,10 +9085,10 @@
         <v>5.5</v>
       </c>
       <c r="L78" s="6"/>
-      <c r="M78" s="192" t="s">
+      <c r="M78" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N78" s="193" t="s">
+      <c r="N78" s="183" t="s">
         <v>818</v>
       </c>
     </row>
@@ -9121,10 +9121,10 @@
         <v>5.5</v>
       </c>
       <c r="L79" s="6"/>
-      <c r="M79" s="192" t="s">
+      <c r="M79" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N79" s="193" t="s">
+      <c r="N79" s="183" t="s">
         <v>786</v>
       </c>
     </row>
@@ -9159,10 +9159,10 @@
         <v>5.5</v>
       </c>
       <c r="L80" s="6"/>
-      <c r="M80" s="192" t="s">
+      <c r="M80" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N80" s="193" t="s">
+      <c r="N80" s="183" t="s">
         <v>818</v>
       </c>
     </row>
@@ -9188,7 +9188,7 @@
       <c r="K81" s="6"/>
       <c r="L81" s="6"/>
       <c r="M81" s="6"/>
-      <c r="N81" s="188"/>
+      <c r="N81" s="178"/>
     </row>
     <row r="82" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="22">
@@ -9221,10 +9221,10 @@
         <v>5.5</v>
       </c>
       <c r="L82" s="6"/>
-      <c r="M82" s="192" t="s">
+      <c r="M82" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N82" s="193" t="s">
+      <c r="N82" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -9252,10 +9252,10 @@
         <f>N83</f>
         <v>Đi chung với với QL.37</v>
       </c>
-      <c r="M83" s="192" t="s">
+      <c r="M83" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N83" s="188" t="s">
+      <c r="N83" s="178" t="s">
         <v>1592</v>
       </c>
     </row>
@@ -9289,10 +9289,10 @@
         <v>5.5</v>
       </c>
       <c r="L84" s="6"/>
-      <c r="M84" s="192" t="s">
+      <c r="M84" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N84" s="193" t="s">
+      <c r="N84" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -9326,10 +9326,10 @@
         <v>9</v>
       </c>
       <c r="L85" s="6"/>
-      <c r="M85" s="192" t="s">
+      <c r="M85" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N85" s="193" t="s">
+      <c r="N85" s="183" t="s">
         <v>810</v>
       </c>
     </row>
@@ -9363,10 +9363,10 @@
         <v>5.5</v>
       </c>
       <c r="L86" s="6"/>
-      <c r="M86" s="192" t="s">
+      <c r="M86" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N86" s="193" t="s">
+      <c r="N86" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -9400,10 +9400,10 @@
         <v>15</v>
       </c>
       <c r="L87" s="6"/>
-      <c r="M87" s="192" t="s">
+      <c r="M87" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N87" s="193" t="s">
+      <c r="N87" s="183" t="s">
         <v>827</v>
       </c>
     </row>
@@ -9437,10 +9437,10 @@
         <v>5.5</v>
       </c>
       <c r="L88" s="6"/>
-      <c r="M88" s="192" t="s">
+      <c r="M88" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N88" s="193" t="s">
+      <c r="N88" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -9474,10 +9474,10 @@
         <v>8</v>
       </c>
       <c r="L89" s="6"/>
-      <c r="M89" s="192" t="s">
+      <c r="M89" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N89" s="193" t="s">
+      <c r="N89" s="183" t="s">
         <v>830</v>
       </c>
     </row>
@@ -9511,10 +9511,10 @@
         <v>5.5</v>
       </c>
       <c r="L90" s="6"/>
-      <c r="M90" s="192" t="s">
+      <c r="M90" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N90" s="193" t="s">
+      <c r="N90" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -9548,10 +9548,10 @@
         <v>9</v>
       </c>
       <c r="L91" s="6"/>
-      <c r="M91" s="192" t="s">
+      <c r="M91" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N91" s="193" t="s">
+      <c r="N91" s="183" t="s">
         <v>810</v>
       </c>
     </row>
@@ -9585,10 +9585,10 @@
         <v>5.5</v>
       </c>
       <c r="L92" s="6"/>
-      <c r="M92" s="192" t="s">
+      <c r="M92" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N92" s="193" t="s">
+      <c r="N92" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -9622,10 +9622,10 @@
         <v>9</v>
       </c>
       <c r="L93" s="6"/>
-      <c r="M93" s="192" t="s">
+      <c r="M93" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N93" s="193" t="s">
+      <c r="N93" s="183" t="s">
         <v>810</v>
       </c>
     </row>
@@ -9659,10 +9659,10 @@
         <v>5.5</v>
       </c>
       <c r="L94" s="6"/>
-      <c r="M94" s="192" t="s">
+      <c r="M94" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N94" s="193" t="s">
+      <c r="N94" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -9696,10 +9696,10 @@
         <v>9</v>
       </c>
       <c r="L95" s="6"/>
-      <c r="M95" s="192" t="s">
+      <c r="M95" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N95" s="193" t="s">
+      <c r="N95" s="183" t="s">
         <v>810</v>
       </c>
     </row>
@@ -9733,10 +9733,10 @@
         <v>5.5</v>
       </c>
       <c r="L96" s="6"/>
-      <c r="M96" s="192" t="s">
+      <c r="M96" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N96" s="193" t="s">
+      <c r="N96" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -9770,10 +9770,10 @@
         <v>9</v>
       </c>
       <c r="L97" s="6"/>
-      <c r="M97" s="192" t="s">
+      <c r="M97" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N97" s="193" t="s">
+      <c r="N97" s="183" t="s">
         <v>810</v>
       </c>
     </row>
@@ -9807,10 +9807,10 @@
         <v>5.5</v>
       </c>
       <c r="L98" s="6"/>
-      <c r="M98" s="192" t="s">
+      <c r="M98" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N98" s="193" t="s">
+      <c r="N98" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -9844,10 +9844,10 @@
         <v>9</v>
       </c>
       <c r="L99" s="6"/>
-      <c r="M99" s="192" t="s">
+      <c r="M99" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N99" s="193" t="s">
+      <c r="N99" s="183" t="s">
         <v>810</v>
       </c>
     </row>
@@ -9881,10 +9881,10 @@
         <v>5.5</v>
       </c>
       <c r="L100" s="6"/>
-      <c r="M100" s="192" t="s">
+      <c r="M100" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N100" s="193" t="s">
+      <c r="N100" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -9918,10 +9918,10 @@
         <v>9</v>
       </c>
       <c r="L101" s="6"/>
-      <c r="M101" s="192" t="s">
+      <c r="M101" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N101" s="193" t="s">
+      <c r="N101" s="183" t="s">
         <v>810</v>
       </c>
     </row>
@@ -9957,10 +9957,10 @@
         <v>5.5</v>
       </c>
       <c r="L102" s="6"/>
-      <c r="M102" s="192" t="s">
+      <c r="M102" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N102" s="193" t="s">
+      <c r="N102" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -9982,7 +9982,7 @@
       <c r="K103" s="6"/>
       <c r="L103" s="6"/>
       <c r="M103" s="6"/>
-      <c r="N103" s="194"/>
+      <c r="N103" s="184"/>
     </row>
     <row r="104" spans="1:14" s="95" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="134" t="s">
@@ -10006,7 +10006,7 @@
       <c r="K104" s="6"/>
       <c r="L104" s="6"/>
       <c r="M104" s="6"/>
-      <c r="N104" s="194"/>
+      <c r="N104" s="184"/>
     </row>
     <row r="105" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="3">
@@ -10039,10 +10039,10 @@
         <v>8</v>
       </c>
       <c r="L105" s="6"/>
-      <c r="M105" s="192" t="s">
+      <c r="M105" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N105" s="189" t="s">
+      <c r="N105" s="179" t="s">
         <v>264</v>
       </c>
     </row>
@@ -10072,7 +10072,7 @@
       <c r="M106" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N106" s="189" t="s">
+      <c r="N106" s="179" t="s">
         <v>167</v>
       </c>
     </row>
@@ -10107,10 +10107,10 @@
         <v>6.5</v>
       </c>
       <c r="L107" s="6"/>
-      <c r="M107" s="192" t="s">
+      <c r="M107" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N107" s="189" t="s">
+      <c r="N107" s="179" t="s">
         <v>263</v>
       </c>
     </row>
@@ -10136,7 +10136,7 @@
       <c r="K108" s="6"/>
       <c r="L108" s="6"/>
       <c r="M108" s="6"/>
-      <c r="N108" s="188"/>
+      <c r="N108" s="178"/>
     </row>
     <row r="109" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="8">
@@ -10169,10 +10169,10 @@
         <v>3.5</v>
       </c>
       <c r="L109" s="6"/>
-      <c r="M109" s="192" t="s">
+      <c r="M109" s="182" t="s">
         <v>1595</v>
       </c>
-      <c r="N109" s="189" t="s">
+      <c r="N109" s="179" t="s">
         <v>262</v>
       </c>
     </row>
@@ -10204,7 +10204,7 @@
       <c r="M110" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N110" s="189" t="s">
+      <c r="N110" s="179" t="s">
         <v>167</v>
       </c>
     </row>
@@ -10230,7 +10230,7 @@
       <c r="K111" s="6"/>
       <c r="L111" s="6"/>
       <c r="M111" s="6"/>
-      <c r="N111" s="188"/>
+      <c r="N111" s="178"/>
     </row>
     <row r="112" spans="1:14" s="18" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="22">
@@ -10266,7 +10266,7 @@
       <c r="M112" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N112" s="193" t="s">
+      <c r="N112" s="183" t="s">
         <v>294</v>
       </c>
     </row>
@@ -10302,7 +10302,7 @@
       <c r="M113" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N113" s="189" t="s">
+      <c r="N113" s="179" t="s">
         <v>295</v>
       </c>
     </row>
@@ -10334,7 +10334,7 @@
       <c r="M114" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N114" s="189" t="s">
+      <c r="N114" s="179" t="s">
         <v>167</v>
       </c>
     </row>
@@ -10360,7 +10360,7 @@
       <c r="K115" s="6"/>
       <c r="L115" s="6"/>
       <c r="M115" s="6"/>
-      <c r="N115" s="188"/>
+      <c r="N115" s="178"/>
     </row>
     <row r="116" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="8">
@@ -10394,7 +10394,7 @@
       <c r="M116" s="6" t="s">
         <v>1597</v>
       </c>
-      <c r="N116" s="189" t="s">
+      <c r="N116" s="179" t="s">
         <v>1572</v>
       </c>
     </row>
@@ -10432,7 +10432,7 @@
       <c r="M117" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N117" s="189" t="s">
+      <c r="N117" s="179" t="s">
         <v>287</v>
       </c>
     </row>
@@ -10468,7 +10468,7 @@
       <c r="M118" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N118" s="189" t="s">
+      <c r="N118" s="179" t="s">
         <v>289</v>
       </c>
     </row>
@@ -10504,7 +10504,7 @@
       <c r="M119" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N119" s="189" t="s">
+      <c r="N119" s="179" t="s">
         <v>291</v>
       </c>
     </row>
@@ -10542,7 +10542,7 @@
       <c r="M120" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N120" s="189" t="s">
+      <c r="N120" s="179" t="s">
         <v>293</v>
       </c>
     </row>
@@ -10566,7 +10566,7 @@
       <c r="K121" s="6"/>
       <c r="L121" s="6"/>
       <c r="M121" s="6"/>
-      <c r="N121" s="188"/>
+      <c r="N121" s="178"/>
     </row>
     <row r="122" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="14">
@@ -10596,7 +10596,7 @@
       <c r="M122" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N122" s="192" t="s">
+      <c r="N122" s="182" t="s">
         <v>167</v>
       </c>
     </row>
@@ -10626,7 +10626,7 @@
       <c r="M123" s="6" t="s">
         <v>1598</v>
       </c>
-      <c r="N123" s="192" t="s">
+      <c r="N123" s="182" t="s">
         <v>300</v>
       </c>
     </row>
@@ -10666,7 +10666,7 @@
       <c r="M124" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N124" s="189" t="s">
+      <c r="N124" s="179" t="s">
         <v>302</v>
       </c>
     </row>
@@ -10692,7 +10692,7 @@
       <c r="K125" s="6"/>
       <c r="L125" s="6"/>
       <c r="M125" s="6"/>
-      <c r="N125" s="188"/>
+      <c r="N125" s="178"/>
     </row>
     <row r="126" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="9">
@@ -10726,7 +10726,7 @@
       <c r="M126" s="6" t="s">
         <v>1599</v>
       </c>
-      <c r="N126" s="192" t="s">
+      <c r="N126" s="182" t="s">
         <v>315</v>
       </c>
     </row>
@@ -10759,7 +10759,7 @@
       <c r="M127" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N127" s="200" t="s">
+      <c r="N127" s="190" t="s">
         <v>1589</v>
       </c>
     </row>
@@ -10793,7 +10793,7 @@
       <c r="M128" s="6" t="s">
         <v>1599</v>
       </c>
-      <c r="N128" s="192" t="s">
+      <c r="N128" s="182" t="s">
         <v>315</v>
       </c>
     </row>
@@ -10831,7 +10831,7 @@
       <c r="M129" s="6" t="s">
         <v>1597</v>
       </c>
-      <c r="N129" s="192" t="s">
+      <c r="N129" s="182" t="s">
         <v>319</v>
       </c>
     </row>
@@ -10857,7 +10857,7 @@
       <c r="K130" s="6"/>
       <c r="L130" s="6"/>
       <c r="M130" s="6"/>
-      <c r="N130" s="188"/>
+      <c r="N130" s="178"/>
     </row>
     <row r="131" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="9">
@@ -10891,7 +10891,7 @@
       <c r="M131" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N131" s="189" t="s">
+      <c r="N131" s="179" t="s">
         <v>167</v>
       </c>
     </row>
@@ -10927,7 +10927,7 @@
       <c r="M132" s="6" t="s">
         <v>1597</v>
       </c>
-      <c r="N132" s="189" t="s">
+      <c r="N132" s="179" t="s">
         <v>266</v>
       </c>
     </row>
@@ -10963,7 +10963,7 @@
       <c r="M133" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N133" s="189" t="s">
+      <c r="N133" s="179" t="s">
         <v>845</v>
       </c>
     </row>
@@ -10999,7 +10999,7 @@
       <c r="M134" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N134" s="189" t="s">
+      <c r="N134" s="179" t="s">
         <v>846</v>
       </c>
     </row>
@@ -11033,7 +11033,7 @@
       <c r="M135" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N135" s="189" t="s">
+      <c r="N135" s="179" t="s">
         <v>167</v>
       </c>
     </row>
@@ -11071,7 +11071,7 @@
       <c r="M136" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N136" s="189" t="s">
+      <c r="N136" s="179" t="s">
         <v>847</v>
       </c>
     </row>
@@ -11097,7 +11097,7 @@
       <c r="K137" s="6"/>
       <c r="L137" s="6"/>
       <c r="M137" s="6"/>
-      <c r="N137" s="188"/>
+      <c r="N137" s="178"/>
     </row>
     <row r="138" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="8">
@@ -11131,7 +11131,7 @@
       <c r="M138" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N138" s="192" t="s">
+      <c r="N138" s="182" t="s">
         <v>167</v>
       </c>
     </row>
@@ -11167,7 +11167,7 @@
       <c r="M139" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N139" s="189" t="s">
+      <c r="N139" s="179" t="s">
         <v>262</v>
       </c>
     </row>
@@ -11198,7 +11198,7 @@
       <c r="M140" s="163" t="s">
         <v>1595</v>
       </c>
-      <c r="N140" s="188" t="s">
+      <c r="N140" s="178" t="s">
         <v>1593</v>
       </c>
     </row>
@@ -11234,45 +11234,45 @@
       <c r="M141" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N141" s="189" t="s">
+      <c r="N141" s="179" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="142" spans="1:14" s="210" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A142" s="201">
+    <row r="142" spans="1:14" s="200" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A142" s="191">
         <v>5</v>
       </c>
-      <c r="B142" s="202" t="s">
+      <c r="B142" s="192" t="s">
         <v>1163</v>
       </c>
-      <c r="C142" s="203" t="s">
+      <c r="C142" s="193" t="s">
         <v>1443</v>
       </c>
-      <c r="D142" s="204" t="s">
+      <c r="D142" s="194" t="s">
         <v>1444</v>
       </c>
-      <c r="E142" s="205">
+      <c r="E142" s="195">
         <v>2023</v>
       </c>
-      <c r="F142" s="206"/>
-      <c r="G142" s="206" t="s">
+      <c r="F142" s="196"/>
+      <c r="G142" s="196" t="s">
         <v>1202</v>
       </c>
-      <c r="H142" s="207"/>
-      <c r="I142" s="207">
+      <c r="H142" s="197"/>
+      <c r="I142" s="197">
         <v>20.8</v>
       </c>
-      <c r="J142" s="208">
+      <c r="J142" s="198">
         <v>6.5</v>
       </c>
-      <c r="K142" s="204">
+      <c r="K142" s="194">
         <v>6.5</v>
       </c>
-      <c r="L142" s="204"/>
-      <c r="M142" s="204" t="s">
+      <c r="L142" s="194"/>
+      <c r="M142" s="194" t="s">
         <v>1595</v>
       </c>
-      <c r="N142" s="209" t="s">
+      <c r="N142" s="199" t="s">
         <v>306</v>
       </c>
     </row>
@@ -11296,7 +11296,7 @@
       <c r="K143" s="6"/>
       <c r="L143" s="6"/>
       <c r="M143" s="6"/>
-      <c r="N143" s="188"/>
+      <c r="N143" s="178"/>
     </row>
     <row r="144" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A144" s="8">
@@ -11326,7 +11326,7 @@
       <c r="M144" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N144" s="192" t="s">
+      <c r="N144" s="182" t="s">
         <v>283</v>
       </c>
     </row>
@@ -11364,7 +11364,7 @@
       <c r="M145" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N145" s="189" t="s">
+      <c r="N145" s="179" t="s">
         <v>262</v>
       </c>
     </row>
@@ -11390,7 +11390,7 @@
       <c r="K146" s="6"/>
       <c r="L146" s="6"/>
       <c r="M146" s="6"/>
-      <c r="N146" s="188"/>
+      <c r="N146" s="178"/>
     </row>
     <row r="147" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="8">
@@ -11426,7 +11426,7 @@
       <c r="M147" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N147" s="189" t="s">
+      <c r="N147" s="179" t="s">
         <v>849</v>
       </c>
     </row>
@@ -11464,7 +11464,7 @@
       <c r="M148" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N148" s="189" t="s">
+      <c r="N148" s="179" t="s">
         <v>845</v>
       </c>
     </row>
@@ -11490,7 +11490,7 @@
       <c r="K149" s="6"/>
       <c r="L149" s="6"/>
       <c r="M149" s="6"/>
-      <c r="N149" s="188"/>
+      <c r="N149" s="178"/>
     </row>
     <row r="150" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="9">
@@ -11526,7 +11526,7 @@
       <c r="M150" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N150" s="189" t="s">
+      <c r="N150" s="179" t="s">
         <v>333</v>
       </c>
     </row>
@@ -11562,7 +11562,7 @@
       <c r="M151" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N151" s="189" t="s">
+      <c r="N151" s="179" t="s">
         <v>334</v>
       </c>
     </row>
@@ -11592,7 +11592,7 @@
       <c r="M152" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N152" s="189" t="s">
+      <c r="N152" s="179" t="s">
         <v>275</v>
       </c>
     </row>
@@ -11628,7 +11628,7 @@
       <c r="M153" s="6" t="s">
         <v>1597</v>
       </c>
-      <c r="N153" s="189" t="s">
+      <c r="N153" s="179" t="s">
         <v>266</v>
       </c>
     </row>
@@ -11660,7 +11660,7 @@
       <c r="M154" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N154" s="189" t="s">
+      <c r="N154" s="179" t="s">
         <v>275</v>
       </c>
     </row>
@@ -11686,7 +11686,7 @@
       <c r="K155" s="6"/>
       <c r="L155" s="6"/>
       <c r="M155" s="6"/>
-      <c r="N155" s="188"/>
+      <c r="N155" s="178"/>
     </row>
     <row r="156" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="8">
@@ -11722,7 +11722,7 @@
       <c r="M156" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N156" s="189" t="s">
+      <c r="N156" s="179" t="s">
         <v>262</v>
       </c>
     </row>
@@ -11758,7 +11758,7 @@
       <c r="M157" s="6" t="s">
         <v>1597</v>
       </c>
-      <c r="N157" s="189" t="s">
+      <c r="N157" s="179" t="s">
         <v>309</v>
       </c>
     </row>
@@ -11788,7 +11788,7 @@
       <c r="M158" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N158" s="192" t="s">
+      <c r="N158" s="182" t="s">
         <v>167</v>
       </c>
     </row>
@@ -11824,7 +11824,7 @@
       <c r="M159" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N159" s="189" t="s">
+      <c r="N159" s="179" t="s">
         <v>312</v>
       </c>
     </row>
@@ -11856,7 +11856,7 @@
       <c r="M160" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N160" s="192" t="s">
+      <c r="N160" s="182" t="s">
         <v>167</v>
       </c>
     </row>
@@ -11882,7 +11882,7 @@
       <c r="K161" s="6"/>
       <c r="L161" s="6"/>
       <c r="M161" s="6"/>
-      <c r="N161" s="188"/>
+      <c r="N161" s="178"/>
     </row>
     <row r="162" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A162" s="8">
@@ -11912,7 +11912,7 @@
       <c r="M162" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N162" s="192" t="s">
+      <c r="N162" s="182" t="s">
         <v>315</v>
       </c>
     </row>
@@ -11945,7 +11945,7 @@
       <c r="M163" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N163" s="200" t="s">
+      <c r="N163" s="190" t="s">
         <v>1590</v>
       </c>
     </row>
@@ -11975,7 +11975,7 @@
       <c r="M164" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N164" s="192" t="s">
+      <c r="N164" s="182" t="s">
         <v>315</v>
       </c>
     </row>
@@ -12011,7 +12011,7 @@
       <c r="M165" s="6" t="s">
         <v>1597</v>
       </c>
-      <c r="N165" s="192" t="s">
+      <c r="N165" s="182" t="s">
         <v>319</v>
       </c>
     </row>
@@ -12041,7 +12041,7 @@
       <c r="M166" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N166" s="192" t="s">
+      <c r="N166" s="182" t="s">
         <v>315</v>
       </c>
     </row>
@@ -12077,7 +12077,7 @@
       <c r="M167" s="6" t="s">
         <v>1597</v>
       </c>
-      <c r="N167" s="192" t="s">
+      <c r="N167" s="182" t="s">
         <v>319</v>
       </c>
     </row>
@@ -12111,7 +12111,7 @@
       <c r="M168" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N168" s="189" t="s">
+      <c r="N168" s="179" t="s">
         <v>331</v>
       </c>
     </row>
@@ -12144,7 +12144,7 @@
       <c r="M169" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N169" s="200" t="s">
+      <c r="N169" s="190" t="s">
         <v>1589</v>
       </c>
     </row>
@@ -12177,7 +12177,7 @@
       <c r="M170" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N170" s="200" t="s">
+      <c r="N170" s="190" t="s">
         <v>1590</v>
       </c>
     </row>
@@ -12213,7 +12213,7 @@
       <c r="M171" s="6" t="s">
         <v>1597</v>
       </c>
-      <c r="N171" s="192" t="s">
+      <c r="N171" s="182" t="s">
         <v>319</v>
       </c>
     </row>
@@ -12249,7 +12249,7 @@
       <c r="M172" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N172" s="189" t="s">
+      <c r="N172" s="179" t="s">
         <v>332</v>
       </c>
     </row>
@@ -12275,7 +12275,7 @@
       <c r="K173" s="6"/>
       <c r="L173" s="6"/>
       <c r="M173" s="6"/>
-      <c r="N173" s="188"/>
+      <c r="N173" s="178"/>
     </row>
     <row r="174" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A174" s="8">
@@ -12305,7 +12305,7 @@
       <c r="M174" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N174" s="192" t="s">
+      <c r="N174" s="182" t="s">
         <v>167</v>
       </c>
     </row>
@@ -12341,7 +12341,7 @@
       <c r="M175" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N175" s="189" t="s">
+      <c r="N175" s="179" t="s">
         <v>346</v>
       </c>
     </row>
@@ -12377,7 +12377,7 @@
       <c r="M176" s="6" t="s">
         <v>1597</v>
       </c>
-      <c r="N176" s="189" t="s">
+      <c r="N176" s="179" t="s">
         <v>319</v>
       </c>
     </row>
@@ -12413,7 +12413,7 @@
       <c r="M177" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N177" s="189" t="s">
+      <c r="N177" s="179" t="s">
         <v>347</v>
       </c>
     </row>
@@ -12443,7 +12443,7 @@
       <c r="M178" s="12" t="s">
         <v>1596</v>
       </c>
-      <c r="N178" s="195" t="s">
+      <c r="N178" s="185" t="s">
         <v>167</v>
       </c>
     </row>
@@ -12474,7 +12474,7 @@
       <c r="M179" s="163" t="s">
         <v>1595</v>
       </c>
-      <c r="N179" s="200" t="s">
+      <c r="N179" s="190" t="s">
         <v>1591</v>
       </c>
     </row>
@@ -12504,7 +12504,7 @@
       <c r="M180" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N180" s="192" t="s">
+      <c r="N180" s="182" t="s">
         <v>167</v>
       </c>
     </row>
@@ -12540,7 +12540,7 @@
       <c r="M181" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N181" s="189" t="s">
+      <c r="N181" s="179" t="s">
         <v>345</v>
       </c>
     </row>
@@ -12570,7 +12570,7 @@
       <c r="M182" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N182" s="192" t="s">
+      <c r="N182" s="182" t="s">
         <v>167</v>
       </c>
     </row>
@@ -12608,7 +12608,7 @@
       <c r="M183" s="6" t="s">
         <v>1597</v>
       </c>
-      <c r="N183" s="189" t="s">
+      <c r="N183" s="179" t="s">
         <v>319</v>
       </c>
     </row>
@@ -12634,7 +12634,7 @@
       <c r="K184" s="6"/>
       <c r="L184" s="6"/>
       <c r="M184" s="6"/>
-      <c r="N184" s="188"/>
+      <c r="N184" s="178"/>
     </row>
     <row r="185" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A185" s="8">
@@ -12666,7 +12666,7 @@
       <c r="M185" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N185" s="192" t="s">
+      <c r="N185" s="182" t="s">
         <v>167</v>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       <c r="M186" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N186" s="189" t="s">
+      <c r="N186" s="179" t="s">
         <v>279</v>
       </c>
     </row>
@@ -12738,7 +12738,7 @@
       <c r="M187" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N187" s="189" t="s">
+      <c r="N187" s="179" t="s">
         <v>1070</v>
       </c>
     </row>
@@ -12774,7 +12774,7 @@
       <c r="M188" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N188" s="189" t="s">
+      <c r="N188" s="179" t="s">
         <v>279</v>
       </c>
     </row>
@@ -12812,7 +12812,7 @@
       <c r="M189" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N189" s="189" t="s">
+      <c r="N189" s="179" t="s">
         <v>279</v>
       </c>
     </row>
@@ -12838,7 +12838,7 @@
       <c r="K190" s="6"/>
       <c r="L190" s="6"/>
       <c r="M190" s="6"/>
-      <c r="N190" s="188"/>
+      <c r="N190" s="178"/>
     </row>
     <row r="191" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A191" s="8">
@@ -12874,7 +12874,7 @@
       <c r="M191" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N191" s="189" t="s">
+      <c r="N191" s="179" t="s">
         <v>278</v>
       </c>
     </row>
@@ -12905,7 +12905,7 @@
       <c r="M192" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N192" s="188" t="s">
+      <c r="N192" s="178" t="s">
         <v>1586</v>
       </c>
     </row>
@@ -12943,7 +12943,7 @@
       <c r="M193" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N193" s="189" t="s">
+      <c r="N193" s="179" t="s">
         <v>279</v>
       </c>
     </row>
@@ -12969,7 +12969,7 @@
       <c r="K194" s="6"/>
       <c r="L194" s="6"/>
       <c r="M194" s="6"/>
-      <c r="N194" s="194"/>
+      <c r="N194" s="184"/>
     </row>
     <row r="195" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A195" s="20">
@@ -13005,7 +13005,7 @@
       <c r="M195" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N195" s="193" t="s">
+      <c r="N195" s="183" t="s">
         <v>278</v>
       </c>
     </row>
@@ -13041,7 +13041,7 @@
       <c r="M196" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N196" s="193" t="s">
+      <c r="N196" s="183" t="s">
         <v>711</v>
       </c>
     </row>
@@ -13079,7 +13079,7 @@
       <c r="M197" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N197" s="193" t="s">
+      <c r="N197" s="183" t="s">
         <v>713</v>
       </c>
     </row>
@@ -13105,7 +13105,7 @@
       <c r="K198" s="6"/>
       <c r="L198" s="6"/>
       <c r="M198" s="6"/>
-      <c r="N198" s="188"/>
+      <c r="N198" s="178"/>
     </row>
     <row r="199" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A199" s="22">
@@ -13143,7 +13143,7 @@
       <c r="M199" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N199" s="193" t="s">
+      <c r="N199" s="183" t="s">
         <v>715</v>
       </c>
     </row>
@@ -13169,7 +13169,7 @@
       <c r="K200" s="6"/>
       <c r="L200" s="6"/>
       <c r="M200" s="6"/>
-      <c r="N200" s="188"/>
+      <c r="N200" s="178"/>
     </row>
     <row r="201" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A201" s="22">
@@ -13205,7 +13205,7 @@
       <c r="M201" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N201" s="193" t="s">
+      <c r="N201" s="183" t="s">
         <v>717</v>
       </c>
     </row>
@@ -13243,7 +13243,7 @@
       <c r="M202" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N202" s="193" t="s">
+      <c r="N202" s="183" t="s">
         <v>1166</v>
       </c>
     </row>
@@ -13269,7 +13269,7 @@
       <c r="K203" s="6"/>
       <c r="L203" s="6"/>
       <c r="M203" s="6"/>
-      <c r="N203" s="188"/>
+      <c r="N203" s="178"/>
     </row>
     <row r="204" spans="1:14" s="18" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A204" s="22">
@@ -13305,7 +13305,7 @@
       <c r="M204" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N204" s="193" t="s">
+      <c r="N204" s="183" t="s">
         <v>295</v>
       </c>
     </row>
@@ -13336,7 +13336,7 @@
       <c r="M205" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N205" s="193" t="s">
+      <c r="N205" s="183" t="s">
         <v>167</v>
       </c>
     </row>
@@ -13372,7 +13372,7 @@
       <c r="M206" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N206" s="193" t="s">
+      <c r="N206" s="183" t="s">
         <v>722</v>
       </c>
     </row>
@@ -13406,7 +13406,7 @@
       <c r="M207" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N207" s="193" t="s">
+      <c r="N207" s="183" t="s">
         <v>167</v>
       </c>
     </row>
@@ -13432,7 +13432,7 @@
       <c r="K208" s="6"/>
       <c r="L208" s="6"/>
       <c r="M208" s="6"/>
-      <c r="N208" s="188"/>
+      <c r="N208" s="178"/>
     </row>
     <row r="209" spans="1:17" s="19" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A209" s="22">
@@ -13468,7 +13468,7 @@
       <c r="M209" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N209" s="193" t="s">
+      <c r="N209" s="183" t="s">
         <v>725</v>
       </c>
     </row>
@@ -13504,7 +13504,7 @@
       <c r="M210" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N210" s="193" t="s">
+      <c r="N210" s="183" t="s">
         <v>727</v>
       </c>
       <c r="Q210" s="116"/>
@@ -13541,7 +13541,7 @@
       <c r="M211" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N211" s="193" t="s">
+      <c r="N211" s="183" t="s">
         <v>729</v>
       </c>
       <c r="Q211" s="116"/>
@@ -13578,7 +13578,7 @@
       <c r="M212" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N212" s="193" t="s">
+      <c r="N212" s="183" t="s">
         <v>711</v>
       </c>
       <c r="Q212" s="116"/>
@@ -13617,7 +13617,7 @@
       <c r="M213" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N213" s="193" t="s">
+      <c r="N213" s="183" t="s">
         <v>732</v>
       </c>
     </row>
@@ -13653,7 +13653,7 @@
       <c r="M214" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N214" s="193" t="s">
+      <c r="N214" s="183" t="s">
         <v>734</v>
       </c>
     </row>
@@ -13679,7 +13679,7 @@
       <c r="K215" s="6"/>
       <c r="L215" s="6"/>
       <c r="M215" s="6"/>
-      <c r="N215" s="188"/>
+      <c r="N215" s="178"/>
     </row>
     <row r="216" spans="1:17" s="19" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A216" s="24">
@@ -13715,7 +13715,7 @@
       <c r="M216" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N216" s="193" t="s">
+      <c r="N216" s="183" t="s">
         <v>736</v>
       </c>
     </row>
@@ -13751,7 +13751,7 @@
       <c r="M217" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N217" s="193" t="s">
+      <c r="N217" s="183" t="s">
         <v>711</v>
       </c>
     </row>
@@ -13787,7 +13787,7 @@
       <c r="M218" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N218" s="193" t="s">
+      <c r="N218" s="183" t="s">
         <v>739</v>
       </c>
     </row>
@@ -13823,7 +13823,7 @@
       <c r="M219" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N219" s="193" t="s">
+      <c r="N219" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -13861,7 +13861,7 @@
       <c r="M220" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N220" s="193" t="s">
+      <c r="N220" s="183" t="s">
         <v>718</v>
       </c>
     </row>
@@ -13886,7 +13886,7 @@
       <c r="K221" s="6"/>
       <c r="L221" s="6"/>
       <c r="M221" s="6"/>
-      <c r="N221" s="188"/>
+      <c r="N221" s="178"/>
     </row>
     <row r="222" spans="1:17" s="19" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A222" s="24">
@@ -13924,7 +13924,7 @@
       <c r="M222" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N222" s="193" t="s">
+      <c r="N222" s="183" t="s">
         <v>743</v>
       </c>
     </row>
@@ -13948,7 +13948,7 @@
       <c r="K223" s="6"/>
       <c r="L223" s="6"/>
       <c r="M223" s="6"/>
-      <c r="N223" s="188"/>
+      <c r="N223" s="178"/>
     </row>
     <row r="224" spans="1:17" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A224" s="22">
@@ -13984,7 +13984,7 @@
       <c r="M224" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N224" s="193" t="s">
+      <c r="N224" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -14021,7 +14021,7 @@
       <c r="M225" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N225" s="193" t="s">
+      <c r="N225" s="183" t="s">
         <v>746</v>
       </c>
     </row>
@@ -14060,7 +14060,7 @@
       <c r="M226" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N226" s="193" t="s">
+      <c r="N226" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -14086,7 +14086,7 @@
       <c r="K227" s="6"/>
       <c r="L227" s="6"/>
       <c r="M227" s="6"/>
-      <c r="N227" s="188"/>
+      <c r="N227" s="178"/>
     </row>
     <row r="228" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A228" s="22">
@@ -14122,7 +14122,7 @@
       <c r="M228" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N228" s="193" t="s">
+      <c r="N228" s="183" t="s">
         <v>749</v>
       </c>
     </row>
@@ -14159,7 +14159,7 @@
       <c r="M229" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N229" s="193" t="s">
+      <c r="N229" s="183" t="s">
         <v>751</v>
       </c>
     </row>
@@ -14196,7 +14196,7 @@
       <c r="M230" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N230" s="193" t="s">
+      <c r="N230" s="183" t="s">
         <v>753</v>
       </c>
     </row>
@@ -14235,7 +14235,7 @@
       <c r="M231" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N231" s="193" t="s">
+      <c r="N231" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -14261,7 +14261,7 @@
       <c r="K232" s="6"/>
       <c r="L232" s="6"/>
       <c r="M232" s="6"/>
-      <c r="N232" s="188"/>
+      <c r="N232" s="178"/>
     </row>
     <row r="233" spans="1:14" s="19" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A233" s="22">
@@ -14297,7 +14297,7 @@
       <c r="M233" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N233" s="193" t="s">
+      <c r="N233" s="183" t="s">
         <v>756</v>
       </c>
     </row>
@@ -14331,7 +14331,7 @@
       <c r="M234" s="6" t="s">
         <v>1596</v>
       </c>
-      <c r="N234" s="193" t="s">
+      <c r="N234" s="183" t="s">
         <v>167</v>
       </c>
     </row>
@@ -14357,7 +14357,7 @@
       <c r="K235" s="6"/>
       <c r="L235" s="6"/>
       <c r="M235" s="6"/>
-      <c r="N235" s="188"/>
+      <c r="N235" s="178"/>
     </row>
     <row r="236" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A236" s="22">
@@ -14395,7 +14395,7 @@
       <c r="M236" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N236" s="193" t="s">
+      <c r="N236" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -14417,7 +14417,7 @@
       <c r="K237" s="6"/>
       <c r="L237" s="6"/>
       <c r="M237" s="6"/>
-      <c r="N237" s="194"/>
+      <c r="N237" s="184"/>
     </row>
     <row r="238" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A238" s="131" t="s">
@@ -14439,7 +14439,7 @@
       <c r="K238" s="6"/>
       <c r="L238" s="6"/>
       <c r="M238" s="6"/>
-      <c r="N238" s="188"/>
+      <c r="N238" s="178"/>
     </row>
     <row r="239" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A239" s="22">
@@ -14475,7 +14475,7 @@
       <c r="M239" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N239" s="193" t="s">
+      <c r="N239" s="183" t="s">
         <v>760</v>
       </c>
     </row>
@@ -14513,7 +14513,7 @@
       <c r="M240" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N240" s="193" t="s">
+      <c r="N240" s="183" t="s">
         <v>746</v>
       </c>
     </row>
@@ -14537,7 +14537,7 @@
       <c r="K241" s="6"/>
       <c r="L241" s="6"/>
       <c r="M241" s="6"/>
-      <c r="N241" s="188"/>
+      <c r="N241" s="178"/>
     </row>
     <row r="242" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A242" s="22">
@@ -14573,7 +14573,7 @@
       <c r="M242" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N242" s="193" t="s">
+      <c r="N242" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -14605,7 +14605,7 @@
       <c r="M243" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N243" s="188" t="s">
+      <c r="N243" s="178" t="s">
         <v>1587</v>
       </c>
     </row>
@@ -14642,7 +14642,7 @@
       <c r="M244" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N244" s="193" t="s">
+      <c r="N244" s="183" t="s">
         <v>279</v>
       </c>
     </row>
@@ -14681,7 +14681,7 @@
       <c r="M245" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N245" s="193" t="s">
+      <c r="N245" s="183" t="s">
         <v>746</v>
       </c>
     </row>
@@ -14705,7 +14705,7 @@
       <c r="K246" s="6"/>
       <c r="L246" s="6"/>
       <c r="M246" s="6"/>
-      <c r="N246" s="194"/>
+      <c r="N246" s="184"/>
     </row>
     <row r="247" spans="1:14" s="19" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A247" s="20">
@@ -14743,7 +14743,7 @@
       <c r="M247" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N247" s="193" t="s">
+      <c r="N247" s="183" t="s">
         <v>769</v>
       </c>
     </row>
@@ -14767,7 +14767,7 @@
       <c r="K248" s="6"/>
       <c r="L248" s="6"/>
       <c r="M248" s="6"/>
-      <c r="N248" s="188"/>
+      <c r="N248" s="178"/>
     </row>
     <row r="249" spans="1:14" s="19" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A249" s="22">
@@ -14803,7 +14803,7 @@
       <c r="M249" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N249" s="193" t="s">
+      <c r="N249" s="183" t="s">
         <v>771</v>
       </c>
     </row>
@@ -14827,7 +14827,7 @@
       <c r="K250" s="6"/>
       <c r="L250" s="6"/>
       <c r="M250" s="6"/>
-      <c r="N250" s="188"/>
+      <c r="N250" s="178"/>
     </row>
     <row r="251" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A251" s="24">
@@ -14863,7 +14863,7 @@
       <c r="M251" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N251" s="193" t="s">
+      <c r="N251" s="183" t="s">
         <v>774</v>
       </c>
     </row>
@@ -14901,7 +14901,7 @@
       <c r="M252" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N252" s="193" t="s">
+      <c r="N252" s="183" t="s">
         <v>776</v>
       </c>
     </row>
@@ -14925,7 +14925,7 @@
       <c r="K253" s="6"/>
       <c r="L253" s="6"/>
       <c r="M253" s="6"/>
-      <c r="N253" s="188"/>
+      <c r="N253" s="178"/>
     </row>
     <row r="254" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A254" s="24">
@@ -14963,7 +14963,7 @@
       <c r="M254" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N254" s="193" t="s">
+      <c r="N254" s="183" t="s">
         <v>779</v>
       </c>
     </row>
@@ -14987,7 +14987,7 @@
       <c r="K255" s="6"/>
       <c r="L255" s="6"/>
       <c r="M255" s="6"/>
-      <c r="N255" s="188"/>
+      <c r="N255" s="178"/>
     </row>
     <row r="256" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A256" s="24">
@@ -15025,7 +15025,7 @@
       <c r="M256" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N256" s="193" t="s">
+      <c r="N256" s="183" t="s">
         <v>779</v>
       </c>
     </row>
@@ -15049,7 +15049,7 @@
       <c r="K257" s="6"/>
       <c r="L257" s="6"/>
       <c r="M257" s="6"/>
-      <c r="N257" s="188"/>
+      <c r="N257" s="178"/>
     </row>
     <row r="258" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A258" s="24">
@@ -15085,7 +15085,7 @@
       <c r="M258" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N258" s="193" t="s">
+      <c r="N258" s="183" t="s">
         <v>784</v>
       </c>
     </row>
@@ -15123,7 +15123,7 @@
       <c r="M259" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N259" s="193" t="s">
+      <c r="N259" s="183" t="s">
         <v>786</v>
       </c>
     </row>
@@ -15147,7 +15147,7 @@
       <c r="K260" s="6"/>
       <c r="L260" s="6"/>
       <c r="M260" s="6"/>
-      <c r="N260" s="188"/>
+      <c r="N260" s="178"/>
     </row>
     <row r="261" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A261" s="24">
@@ -15181,7 +15181,7 @@
       <c r="M261" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N261" s="193" t="s">
+      <c r="N261" s="183" t="s">
         <v>788</v>
       </c>
     </row>
@@ -15205,7 +15205,7 @@
       <c r="K262" s="6"/>
       <c r="L262" s="6"/>
       <c r="M262" s="6"/>
-      <c r="N262" s="188"/>
+      <c r="N262" s="178"/>
     </row>
     <row r="263" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A263" s="24">
@@ -15239,7 +15239,7 @@
       <c r="M263" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N263" s="193" t="s">
+      <c r="N263" s="183" t="s">
         <v>788</v>
       </c>
     </row>
@@ -15263,7 +15263,7 @@
       <c r="K264" s="6"/>
       <c r="L264" s="6"/>
       <c r="M264" s="6"/>
-      <c r="N264" s="188"/>
+      <c r="N264" s="178"/>
     </row>
     <row r="265" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A265" s="24">
@@ -15299,7 +15299,7 @@
       <c r="M265" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N265" s="193" t="s">
+      <c r="N265" s="183" t="s">
         <v>790</v>
       </c>
     </row>
@@ -15335,7 +15335,7 @@
       <c r="M266" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N266" s="193" t="s">
+      <c r="N266" s="183" t="s">
         <v>790</v>
       </c>
     </row>
@@ -15371,7 +15371,7 @@
       <c r="M267" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N267" s="193" t="s">
+      <c r="N267" s="183" t="s">
         <v>790</v>
       </c>
     </row>
@@ -15409,7 +15409,7 @@
       <c r="M268" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N268" s="193" t="s">
+      <c r="N268" s="183" t="s">
         <v>790</v>
       </c>
     </row>
@@ -15433,7 +15433,7 @@
       <c r="K269" s="6"/>
       <c r="L269" s="6"/>
       <c r="M269" s="6"/>
-      <c r="N269" s="197"/>
+      <c r="N269" s="187"/>
     </row>
     <row r="270" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A270" s="20">
@@ -15471,7 +15471,7 @@
       <c r="M270" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N270" s="198" t="s">
+      <c r="N270" s="188" t="s">
         <v>795</v>
       </c>
     </row>
@@ -15495,7 +15495,7 @@
       <c r="K271" s="6"/>
       <c r="L271" s="6"/>
       <c r="M271" s="6"/>
-      <c r="N271" s="189"/>
+      <c r="N271" s="179"/>
     </row>
     <row r="272" spans="1:14" s="18" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A272" s="22">
@@ -15525,7 +15525,7 @@
       <c r="M272" s="6" t="s">
         <v>1595</v>
       </c>
-      <c r="N272" s="193" t="s">
+      <c r="N272" s="183" t="s">
         <v>1250</v>
       </c>
     </row>
@@ -15557,73 +15557,73 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="177" t="s">
+      <c r="A1" s="201" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="177"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
-      <c r="E1" s="177"/>
-      <c r="F1" s="177"/>
-      <c r="G1" s="177"/>
-      <c r="H1" s="177"/>
-      <c r="I1" s="177"/>
-      <c r="J1" s="177"/>
-      <c r="K1" s="177"/>
+      <c r="B1" s="201"/>
+      <c r="C1" s="201"/>
+      <c r="D1" s="201"/>
+      <c r="E1" s="201"/>
+      <c r="F1" s="201"/>
+      <c r="G1" s="201"/>
+      <c r="H1" s="201"/>
+      <c r="I1" s="201"/>
+      <c r="J1" s="201"/>
+      <c r="K1" s="201"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="178" t="e">
+      <c r="A2" s="202" t="e">
         <f>'Phụ Lục 1'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="B2" s="178"/>
-      <c r="C2" s="178"/>
-      <c r="D2" s="178"/>
-      <c r="E2" s="178"/>
-      <c r="F2" s="178"/>
-      <c r="G2" s="178"/>
-      <c r="H2" s="178"/>
-      <c r="I2" s="178"/>
-      <c r="J2" s="178"/>
-      <c r="K2" s="178"/>
+      <c r="B2" s="202"/>
+      <c r="C2" s="202"/>
+      <c r="D2" s="202"/>
+      <c r="E2" s="202"/>
+      <c r="F2" s="202"/>
+      <c r="G2" s="202"/>
+      <c r="H2" s="202"/>
+      <c r="I2" s="202"/>
+      <c r="J2" s="202"/>
+      <c r="K2" s="202"/>
     </row>
     <row r="4" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="179" t="s">
+      <c r="A4" s="203" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="179" t="s">
+      <c r="B4" s="203" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="180" t="s">
+      <c r="C4" s="204" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="181"/>
-      <c r="E4" s="179" t="s">
+      <c r="D4" s="205"/>
+      <c r="E4" s="203" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="180" t="s">
+      <c r="F4" s="204" t="s">
         <v>348</v>
       </c>
-      <c r="G4" s="181"/>
-      <c r="H4" s="179" t="s">
+      <c r="G4" s="205"/>
+      <c r="H4" s="203" t="s">
         <v>5</v>
       </c>
-      <c r="I4" s="179"/>
-      <c r="J4" s="179"/>
-      <c r="K4" s="179" t="s">
+      <c r="I4" s="203"/>
+      <c r="J4" s="203"/>
+      <c r="K4" s="203" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="179"/>
-      <c r="B5" s="179"/>
+      <c r="A5" s="203"/>
+      <c r="B5" s="203"/>
       <c r="C5" s="16" t="s">
         <v>353</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="E5" s="179"/>
+      <c r="E5" s="203"/>
       <c r="F5" s="15" t="s">
         <v>349</v>
       </c>
@@ -15639,7 +15639,7 @@
       <c r="J5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K5" s="179"/>
+      <c r="K5" s="203"/>
     </row>
     <row r="6" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7">
@@ -17324,60 +17324,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="183" t="s">
+      <c r="A1" s="207" t="s">
         <v>844</v>
       </c>
-      <c r="B1" s="183"/>
-      <c r="C1" s="183"/>
-      <c r="D1" s="183"/>
-      <c r="E1" s="183"/>
-      <c r="F1" s="183"/>
-      <c r="G1" s="183"/>
-      <c r="H1" s="183"/>
-      <c r="I1" s="183"/>
+      <c r="B1" s="207"/>
+      <c r="C1" s="207"/>
+      <c r="D1" s="207"/>
+      <c r="E1" s="207"/>
+      <c r="F1" s="207"/>
+      <c r="G1" s="207"/>
+      <c r="H1" s="207"/>
+      <c r="I1" s="207"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="184" t="e">
+      <c r="A2" s="208" t="e">
         <f>'Phụ Lục 1'!#REF!</f>
         <v>#REF!</v>
       </c>
-      <c r="B2" s="184"/>
-      <c r="C2" s="184"/>
-      <c r="D2" s="184"/>
-      <c r="E2" s="184"/>
-      <c r="F2" s="184"/>
-      <c r="G2" s="184"/>
-      <c r="H2" s="184"/>
-      <c r="I2" s="184"/>
+      <c r="B2" s="208"/>
+      <c r="C2" s="208"/>
+      <c r="D2" s="208"/>
+      <c r="E2" s="208"/>
+      <c r="F2" s="208"/>
+      <c r="G2" s="208"/>
+      <c r="H2" s="208"/>
+      <c r="I2" s="208"/>
     </row>
     <row r="4" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="185" t="s">
+      <c r="A4" s="209" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="185" t="s">
+      <c r="B4" s="209" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="185" t="s">
+      <c r="C4" s="209" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="185" t="s">
+      <c r="D4" s="209" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="185" t="s">
+      <c r="E4" s="209" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="185"/>
-      <c r="G4" s="185"/>
-      <c r="H4" s="185"/>
-      <c r="I4" s="185" t="s">
+      <c r="F4" s="209"/>
+      <c r="G4" s="209"/>
+      <c r="H4" s="209"/>
+      <c r="I4" s="209" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="82.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="185"/>
-      <c r="B5" s="185"/>
-      <c r="C5" s="185"/>
-      <c r="D5" s="185"/>
+      <c r="A5" s="209"/>
+      <c r="B5" s="209"/>
+      <c r="C5" s="209"/>
+      <c r="D5" s="209"/>
       <c r="E5" s="33" t="s">
         <v>9</v>
       </c>
@@ -17390,7 +17390,7 @@
       <c r="H5" s="33" t="s">
         <v>1078</v>
       </c>
-      <c r="I5" s="185"/>
+      <c r="I5" s="209"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="26">
@@ -17425,10 +17425,10 @@
       <c r="A7" s="62" t="s">
         <v>245</v>
       </c>
-      <c r="B7" s="186" t="s">
+      <c r="B7" s="210" t="s">
         <v>565</v>
       </c>
-      <c r="C7" s="186"/>
+      <c r="C7" s="210"/>
       <c r="D7" s="63"/>
       <c r="E7" s="63"/>
       <c r="F7" s="63"/>
@@ -22251,10 +22251,10 @@
       <c r="A190" s="62" t="s">
         <v>564</v>
       </c>
-      <c r="B190" s="186" t="s">
+      <c r="B190" s="210" t="s">
         <v>563</v>
       </c>
-      <c r="C190" s="186"/>
+      <c r="C190" s="210"/>
       <c r="D190" s="63"/>
       <c r="E190" s="63"/>
       <c r="F190" s="63"/>
@@ -27625,56 +27625,56 @@
       </c>
     </row>
     <row r="400" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A400" s="182" t="s">
+      <c r="A400" s="206" t="s">
         <v>1125</v>
       </c>
-      <c r="B400" s="182"/>
-      <c r="C400" s="182"/>
-      <c r="D400" s="182"/>
-      <c r="E400" s="182"/>
-      <c r="F400" s="182"/>
-      <c r="G400" s="182"/>
-      <c r="H400" s="182"/>
-      <c r="I400" s="182"/>
+      <c r="B400" s="206"/>
+      <c r="C400" s="206"/>
+      <c r="D400" s="206"/>
+      <c r="E400" s="206"/>
+      <c r="F400" s="206"/>
+      <c r="G400" s="206"/>
+      <c r="H400" s="206"/>
+      <c r="I400" s="206"/>
     </row>
     <row r="401" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A401" s="182" t="s">
+      <c r="A401" s="206" t="s">
         <v>1126</v>
       </c>
-      <c r="B401" s="182"/>
-      <c r="C401" s="182"/>
-      <c r="D401" s="182"/>
-      <c r="E401" s="182"/>
-      <c r="F401" s="182"/>
-      <c r="G401" s="182"/>
-      <c r="H401" s="182"/>
-      <c r="I401" s="182"/>
+      <c r="B401" s="206"/>
+      <c r="C401" s="206"/>
+      <c r="D401" s="206"/>
+      <c r="E401" s="206"/>
+      <c r="F401" s="206"/>
+      <c r="G401" s="206"/>
+      <c r="H401" s="206"/>
+      <c r="I401" s="206"/>
     </row>
     <row r="402" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A402" s="182" t="s">
+      <c r="A402" s="206" t="s">
         <v>1127</v>
       </c>
-      <c r="B402" s="182"/>
-      <c r="C402" s="182"/>
-      <c r="D402" s="182"/>
-      <c r="E402" s="182"/>
-      <c r="F402" s="182"/>
-      <c r="G402" s="182"/>
-      <c r="H402" s="182"/>
-      <c r="I402" s="182"/>
+      <c r="B402" s="206"/>
+      <c r="C402" s="206"/>
+      <c r="D402" s="206"/>
+      <c r="E402" s="206"/>
+      <c r="F402" s="206"/>
+      <c r="G402" s="206"/>
+      <c r="H402" s="206"/>
+      <c r="I402" s="206"/>
     </row>
     <row r="403" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A403" s="182" t="s">
+      <c r="A403" s="206" t="s">
         <v>355</v>
       </c>
-      <c r="B403" s="182"/>
-      <c r="C403" s="182"/>
-      <c r="D403" s="182"/>
-      <c r="E403" s="182"/>
-      <c r="F403" s="182"/>
-      <c r="G403" s="182"/>
-      <c r="H403" s="182"/>
-      <c r="I403" s="182"/>
+      <c r="B403" s="206"/>
+      <c r="C403" s="206"/>
+      <c r="D403" s="206"/>
+      <c r="E403" s="206"/>
+      <c r="F403" s="206"/>
+      <c r="G403" s="206"/>
+      <c r="H403" s="206"/>
+      <c r="I403" s="206"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>